<commit_message>
Completed Nifty100 Financial Analytics Platform
</commit_message>
<xml_diff>
--- a/output/cashflow_intelligence.xlsx
+++ b/output/cashflow_intelligence.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J101"/>
+  <dimension ref="A1:I101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,11 +462,6 @@
           <t>deleveraging_flag</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>capital_allocation_label</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -502,7 +497,6 @@
       <c r="I2" t="b">
         <v>1</v>
       </c>
-      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -538,7 +532,6 @@
       <c r="I3" t="b">
         <v>0</v>
       </c>
-      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -574,7 +567,6 @@
       <c r="I4" t="b">
         <v>0</v>
       </c>
-      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -610,7 +602,6 @@
       <c r="I5" t="b">
         <v>0</v>
       </c>
-      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -646,7 +637,6 @@
       <c r="I6" t="b">
         <v>1</v>
       </c>
-      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -682,7 +672,6 @@
       <c r="I7" t="b">
         <v>1</v>
       </c>
-      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -718,7 +707,6 @@
       <c r="I8" t="b">
         <v>0</v>
       </c>
-      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -754,7 +742,6 @@
       <c r="I9" t="b">
         <v>0</v>
       </c>
-      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -790,7 +777,6 @@
       <c r="I10" t="b">
         <v>0</v>
       </c>
-      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -818,7 +804,6 @@
       <c r="I11" t="b">
         <v>0</v>
       </c>
-      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -854,7 +839,6 @@
       <c r="I12" t="b">
         <v>0</v>
       </c>
-      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -890,7 +874,6 @@
       <c r="I13" t="b">
         <v>0</v>
       </c>
-      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -926,7 +909,6 @@
       <c r="I14" t="b">
         <v>0</v>
       </c>
-      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -962,7 +944,6 @@
       <c r="I15" t="b">
         <v>1</v>
       </c>
-      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -998,7 +979,6 @@
       <c r="I16" t="b">
         <v>0</v>
       </c>
-      <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1034,7 +1014,6 @@
       <c r="I17" t="b">
         <v>0</v>
       </c>
-      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1070,7 +1049,6 @@
       <c r="I18" t="b">
         <v>0</v>
       </c>
-      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1106,7 +1084,6 @@
       <c r="I19" t="b">
         <v>1</v>
       </c>
-      <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1142,7 +1119,6 @@
       <c r="I20" t="b">
         <v>0</v>
       </c>
-      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1178,7 +1154,6 @@
       <c r="I21" t="b">
         <v>1</v>
       </c>
-      <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1214,7 +1189,6 @@
       <c r="I22" t="b">
         <v>1</v>
       </c>
-      <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1250,7 +1224,6 @@
       <c r="I23" t="b">
         <v>1</v>
       </c>
-      <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1286,7 +1259,6 @@
       <c r="I24" t="b">
         <v>0</v>
       </c>
-      <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1322,7 +1294,6 @@
       <c r="I25" t="b">
         <v>0</v>
       </c>
-      <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1358,7 +1329,6 @@
       <c r="I26" t="b">
         <v>1</v>
       </c>
-      <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1394,7 +1364,6 @@
       <c r="I27" t="b">
         <v>0</v>
       </c>
-      <c r="J27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1430,7 +1399,6 @@
       <c r="I28" t="b">
         <v>0</v>
       </c>
-      <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1466,7 +1434,6 @@
       <c r="I29" t="b">
         <v>1</v>
       </c>
-      <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1502,7 +1469,6 @@
       <c r="I30" t="b">
         <v>0</v>
       </c>
-      <c r="J30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1538,7 +1504,6 @@
       <c r="I31" t="b">
         <v>1</v>
       </c>
-      <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1574,7 +1539,6 @@
       <c r="I32" t="b">
         <v>0</v>
       </c>
-      <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1610,7 +1574,6 @@
       <c r="I33" t="b">
         <v>0</v>
       </c>
-      <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1646,7 +1609,6 @@
       <c r="I34" t="b">
         <v>0</v>
       </c>
-      <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1682,7 +1644,6 @@
       <c r="I35" t="b">
         <v>0</v>
       </c>
-      <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1718,7 +1679,6 @@
       <c r="I36" t="b">
         <v>0</v>
       </c>
-      <c r="J36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1754,7 +1714,6 @@
       <c r="I37" t="b">
         <v>0</v>
       </c>
-      <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1790,7 +1749,6 @@
       <c r="I38" t="b">
         <v>0</v>
       </c>
-      <c r="J38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1826,7 +1784,6 @@
       <c r="I39" t="b">
         <v>0</v>
       </c>
-      <c r="J39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1862,7 +1819,6 @@
       <c r="I40" t="b">
         <v>0</v>
       </c>
-      <c r="J40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1898,7 +1854,6 @@
       <c r="I41" t="b">
         <v>0</v>
       </c>
-      <c r="J41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1934,7 +1889,6 @@
       <c r="I42" t="b">
         <v>0</v>
       </c>
-      <c r="J42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1970,7 +1924,6 @@
       <c r="I43" t="b">
         <v>1</v>
       </c>
-      <c r="J43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2006,7 +1959,6 @@
       <c r="I44" t="b">
         <v>0</v>
       </c>
-      <c r="J44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2042,7 +1994,6 @@
       <c r="I45" t="b">
         <v>0</v>
       </c>
-      <c r="J45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2078,7 +2029,6 @@
       <c r="I46" t="b">
         <v>0</v>
       </c>
-      <c r="J46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2114,7 +2064,6 @@
       <c r="I47" t="b">
         <v>0</v>
       </c>
-      <c r="J47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2150,7 +2099,6 @@
       <c r="I48" t="b">
         <v>0</v>
       </c>
-      <c r="J48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2186,7 +2134,6 @@
       <c r="I49" t="b">
         <v>0</v>
       </c>
-      <c r="J49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2222,7 +2169,6 @@
       <c r="I50" t="b">
         <v>0</v>
       </c>
-      <c r="J50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2258,7 +2204,6 @@
       <c r="I51" t="b">
         <v>1</v>
       </c>
-      <c r="J51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2294,7 +2239,6 @@
       <c r="I52" t="b">
         <v>1</v>
       </c>
-      <c r="J52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2330,7 +2274,6 @@
       <c r="I53" t="b">
         <v>1</v>
       </c>
-      <c r="J53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2366,7 +2309,6 @@
       <c r="I54" t="b">
         <v>1</v>
       </c>
-      <c r="J54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2402,7 +2344,6 @@
       <c r="I55" t="b">
         <v>0</v>
       </c>
-      <c r="J55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2438,7 +2379,6 @@
       <c r="I56" t="b">
         <v>1</v>
       </c>
-      <c r="J56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2474,7 +2414,6 @@
       <c r="I57" t="b">
         <v>0</v>
       </c>
-      <c r="J57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2510,7 +2449,6 @@
       <c r="I58" t="b">
         <v>0</v>
       </c>
-      <c r="J58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2546,7 +2484,6 @@
       <c r="I59" t="b">
         <v>0</v>
       </c>
-      <c r="J59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2582,7 +2519,6 @@
       <c r="I60" t="b">
         <v>0</v>
       </c>
-      <c r="J60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2618,7 +2554,6 @@
       <c r="I61" t="b">
         <v>0</v>
       </c>
-      <c r="J61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2654,7 +2589,6 @@
       <c r="I62" t="b">
         <v>0</v>
       </c>
-      <c r="J62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2690,7 +2624,6 @@
       <c r="I63" t="b">
         <v>0</v>
       </c>
-      <c r="J63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2726,7 +2659,6 @@
       <c r="I64" t="b">
         <v>0</v>
       </c>
-      <c r="J64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2762,7 +2694,6 @@
       <c r="I65" t="b">
         <v>1</v>
       </c>
-      <c r="J65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2798,7 +2729,6 @@
       <c r="I66" t="b">
         <v>0</v>
       </c>
-      <c r="J66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2834,7 +2764,6 @@
       <c r="I67" t="b">
         <v>0</v>
       </c>
-      <c r="J67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2870,7 +2799,6 @@
       <c r="I68" t="b">
         <v>0</v>
       </c>
-      <c r="J68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2906,7 +2834,6 @@
       <c r="I69" t="b">
         <v>0</v>
       </c>
-      <c r="J69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2942,7 +2869,6 @@
       <c r="I70" t="b">
         <v>0</v>
       </c>
-      <c r="J70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2978,7 +2904,6 @@
       <c r="I71" t="b">
         <v>0</v>
       </c>
-      <c r="J71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3014,7 +2939,6 @@
       <c r="I72" t="b">
         <v>0</v>
       </c>
-      <c r="J72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3050,7 +2974,6 @@
       <c r="I73" t="b">
         <v>1</v>
       </c>
-      <c r="J73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3086,7 +3009,6 @@
       <c r="I74" t="b">
         <v>0</v>
       </c>
-      <c r="J74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3122,7 +3044,6 @@
       <c r="I75" t="b">
         <v>1</v>
       </c>
-      <c r="J75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3158,7 +3079,6 @@
       <c r="I76" t="b">
         <v>0</v>
       </c>
-      <c r="J76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3194,7 +3114,6 @@
       <c r="I77" t="b">
         <v>0</v>
       </c>
-      <c r="J77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3230,7 +3149,6 @@
       <c r="I78" t="b">
         <v>0</v>
       </c>
-      <c r="J78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3266,7 +3184,6 @@
       <c r="I79" t="b">
         <v>0</v>
       </c>
-      <c r="J79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3302,7 +3219,6 @@
       <c r="I80" t="b">
         <v>1</v>
       </c>
-      <c r="J80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3338,7 +3254,6 @@
       <c r="I81" t="b">
         <v>0</v>
       </c>
-      <c r="J81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3374,11 +3289,6 @@
       <c r="I82" t="b">
         <v>0</v>
       </c>
-      <c r="J82" t="inlineStr">
-        <is>
-          <t>Reinvestor</t>
-        </is>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3414,7 +3324,6 @@
       <c r="I83" t="b">
         <v>1</v>
       </c>
-      <c r="J83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3450,7 +3359,6 @@
       <c r="I84" t="b">
         <v>0</v>
       </c>
-      <c r="J84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3486,7 +3394,6 @@
       <c r="I85" t="b">
         <v>1</v>
       </c>
-      <c r="J85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3522,7 +3429,6 @@
       <c r="I86" t="b">
         <v>0</v>
       </c>
-      <c r="J86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3558,7 +3464,6 @@
       <c r="I87" t="b">
         <v>0</v>
       </c>
-      <c r="J87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3594,7 +3499,6 @@
       <c r="I88" t="b">
         <v>0</v>
       </c>
-      <c r="J88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3630,7 +3534,6 @@
       <c r="I89" t="b">
         <v>1</v>
       </c>
-      <c r="J89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3666,7 +3569,6 @@
       <c r="I90" t="b">
         <v>0</v>
       </c>
-      <c r="J90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3702,7 +3604,6 @@
       <c r="I91" t="b">
         <v>1</v>
       </c>
-      <c r="J91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3738,7 +3639,6 @@
       <c r="I92" t="b">
         <v>1</v>
       </c>
-      <c r="J92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3774,7 +3674,6 @@
       <c r="I93" t="b">
         <v>0</v>
       </c>
-      <c r="J93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3810,7 +3709,6 @@
       <c r="I94" t="b">
         <v>0</v>
       </c>
-      <c r="J94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3846,7 +3744,6 @@
       <c r="I95" t="b">
         <v>0</v>
       </c>
-      <c r="J95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3882,7 +3779,6 @@
       <c r="I96" t="b">
         <v>0</v>
       </c>
-      <c r="J96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3918,7 +3814,6 @@
       <c r="I97" t="b">
         <v>0</v>
       </c>
-      <c r="J97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3954,7 +3849,6 @@
       <c r="I98" t="b">
         <v>0</v>
       </c>
-      <c r="J98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3990,7 +3884,6 @@
       <c r="I99" t="b">
         <v>0</v>
       </c>
-      <c r="J99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -4026,7 +3919,6 @@
       <c r="I100" t="b">
         <v>0</v>
       </c>
-      <c r="J100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -4062,7 +3954,6 @@
       <c r="I101" t="b">
         <v>0</v>
       </c>
-      <c r="J101" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Improved financial analytics engine and added screener API
</commit_message>
<xml_diff>
--- a/output/cashflow_intelligence.xlsx
+++ b/output/cashflow_intelligence.xlsx
@@ -680,7 +680,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1.470072585366305</v>
+        <v>1.176058068293044</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -784,19 +784,25 @@
           <t>ATGL</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>Accrual Risk</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Capital Intensive</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
+          <t>Asset Light</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="b">
         <v>0</v>

</xml_diff>